<commit_message>
feat(sprint-sync): ingested Day 1 Google Meet Gemini meeting notes into Sprint 1 Daily Log, Excel tracker, and Slack #all-mas-ai-labs
</commit_message>
<xml_diff>
--- a/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
+++ b/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
@@ -461,7 +461,7 @@
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[!] Blocked</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -5696,7 +5696,7 @@
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -5846,7 +5846,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[!] Blocked</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6131,7 +6131,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -6644,7 +6644,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -6758,7 +6758,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: complete dynamic task lifecycle (/add-task, /deprioritize-task) and cloud deployment bundle
</commit_message>
<xml_diff>
--- a/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
+++ b/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -464,7 +464,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
@@ -874,7 +874,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>[!] Blocked</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Need to discuss the artifacts required for capability mapping</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>working on bug hunterz pipeline migrating it to new email and also improving the pipeline</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1221,27 +1221,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
+          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>S1.12</t>
+          <t>S1.22</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Inventory current GCP projects, services &amp; VMs</t>
+          <t>Sales Suite technical documentation &amp; research plan</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Rohan</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 3 (Day 3)</t>
+          <t>Fri, Sept 4 (Day 4)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Complete GCP infrastructure inventory with instance sizes</t>
+          <t>Technical architecture doc &amp; generalized setup plan</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1288,12 +1288,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>S1.13</t>
+          <t>S1.12</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Inventory AWS accounts/services used by AI Labs</t>
+          <t>Inventory current GCP projects, services &amp; VMs</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 4 (Day 4)</t>
+          <t>Thu, Sept 3 (Day 3)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Complete AWS inventory (S3, compute, IAM)</t>
+          <t>Complete GCP infrastructure inventory with instance sizes</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>S1.14</t>
+          <t>S1.13</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Master inventory of AI/API keys, models &amp; endpoints</t>
+          <t>Inventory AWS accounts/services used by AI Labs</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>All third-party AI keys mapped to product modules</t>
+          <t>Complete AWS inventory (S3, compute, IAM)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>S1.15</t>
+          <t>S1.14</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Collect top repetitive workflows across MAS departments</t>
+          <t>Master inventory of AI/API keys, models &amp; endpoints</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Departmental automation intake list (Problem $\rightarrow$ Effort $\rightarrow$ Value)</t>
+          <t>All third-party AI keys mapped to product modules</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1474,32 +1474,32 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>S1.16</t>
+          <t>S1.15</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>**Build &amp; configure MAS Slack Standup Bot v1.0**</t>
+          <t>Collect top repetitive workflows across MAS departments</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Rohan</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>**Thu, Sept 3 (Day 3)**</t>
+          <t>Fri, Sept 4 (Day 4)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>**Personal DMs, dropdown modal, 7:45 PM summary &amp; 2-way sync**</t>
+          <t>Departmental automation intake list (Problem $\rightarrow$ Effort $\rightarrow$ Value)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1536,12 +1536,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>S1.17</t>
+          <t>S1.16</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>**Test &amp; pilot Slack Standup Bot with core team**</t>
+          <t>**Build &amp; configure MAS Slack Standup Bot v1.0**</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>**Fri, Sept 4 (Day 4)**</t>
+          <t>**Thu, Sept 3 (Day 3)**</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>**Live test during Friday standup &amp; Friday review #1**</t>
+          <t>**Personal DMs, dropdown modal, 7:45 PM summary &amp; 2-way sync**</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Need to discuss the artifacts required for capability mapping</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1593,27 +1593,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
+          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>S1.18</t>
+          <t>S1.17</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Kick off QA Tester (contract/2-mo) hiring</t>
+          <t>**Test &amp; pilot Slack Standup Bot with core team**</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Gaurav</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Tue, Sept 1 (Day 1)</t>
+          <t>**Fri, Sept 4 (Day 4)**</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Active job description &amp; candidate pipeline with HR</t>
+          <t>**Live test during Friday standup &amp; Friday review #1**</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Need to discuss the artifacts required for capability mapping</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1660,12 +1660,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>S1.19</t>
+          <t>S1.18</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Kick off PM Intern (25 hrs/wk) hiring</t>
+          <t>Kick off QA Tester (contract/2-mo) hiring</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1680,12 +1680,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Active job description &amp; candidate sourcing</t>
+          <t>Active job description &amp; candidate pipeline with HR</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1722,12 +1722,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>S1.20</t>
+          <t>S1.19</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Initial September GPU/compute sync with Sajan</t>
+          <t>Kick off PM Intern (25 hrs/wk) hiring</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 3 (Day 3)</t>
+          <t>Tue, Sept 1 (Day 1)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Compute vendor contacts &amp; initial workload candidate list</t>
+          <t>Active job description &amp; candidate sourcing</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1784,12 +1784,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>S1.21</t>
+          <t>S1.20</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>**Weekly Product &amp; Capability Review #1 (8:00 PM)**</t>
+          <t>Initial September GPU/compute sync with Sajan</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 4 (Day 4)</t>
+          <t>Thu, Sept 3 (Day 3)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Review minutes, Week 1 bug fix verification &amp; RAG audit</t>
+          <t>Compute vendor contacts &amp; initial workload candidate list</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1836,32 +1836,32 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Compartment 1: Market, Intake &amp; Client POCs</t>
+          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>S2.1</t>
+          <t>S1.21</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Walkthrough Intake Process with Pranab Sir</t>
+          <t>**Weekly Product &amp; Capability Review #1 (8:00 PM)**</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Prakhar</t>
+          <t>Gaurav</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Mon, Sept 7 (Day 7)</t>
+          <t>Fri, Sept 4 (Day 4)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Business alignment on mandatory intake rules</t>
+          <t>Review minutes, Week 1 bug fix verification &amp; RAG audit</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1908,12 +1908,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>S2.2</t>
+          <t>S2.1</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>**Sign off Business $\rightarrow$ Tech Intake Format (M6)**</t>
+          <t>Walkthrough Intake Process with Pranab Sir</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>**Thu, Sept 10 (Day 10)**</t>
+          <t>Mon, Sept 7 (Day 7)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>**Joint intake format signed off; live for Fri, Sept 11**</t>
+          <t>Business alignment on mandatory intake rules</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1970,22 +1970,22 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>S2.3</t>
+          <t>S2.2</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Conduct structured scoping call: **Orane**</t>
+          <t>**Sign off Business $\rightarrow$ Tech Intake Format (M6)**</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Prakhar</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Tue, Sept 8 (Day 8)</t>
+          <t>**Thu, Sept 10 (Day 10)**</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Scope v1 draft for Orane (scale, features, timeline)</t>
+          <t>**Joint intake format signed off; live for Fri, Sept 11**</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>S2.4</t>
+          <t>S2.3</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Conduct structured scoping call: **College Vidya**</t>
+          <t>Conduct structured scoping call: **Orane**</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 9 (Day 9)</t>
+          <t>Tue, Sept 8 (Day 8)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Scope v1 draft for College Vidya (CRM/voice needs)</t>
+          <t>Scope v1 draft for Orane (scale, features, timeline)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2094,12 +2094,12 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>S2.5</t>
+          <t>S2.4</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Conduct structured scoping call: **Chitkara**</t>
+          <t>Conduct structured scoping call: **College Vidya**</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 10 (Day 10)</t>
+          <t>Wed, Sept 9 (Day 9)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Scope v1 draft for Chitkara (100-student placement cohort)</t>
+          <t>Scope v1 draft for College Vidya (CRM/voice needs)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2156,12 +2156,12 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>S2.6</t>
+          <t>S2.5</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Consolidate 3 Client Scope v1 drafts</t>
+          <t>Conduct structured scoping call: **Chitkara**</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 11 (Day 11)</t>
+          <t>Thu, Sept 10 (Day 10)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>3 Scopes ready for technical feasibility review</t>
+          <t>Scope v1 draft for Chitkara (100-student placement cohort)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2218,17 +2218,17 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>S2.7</t>
+          <t>S2.6</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Finalize &amp; format **Product Catalogue v1**</t>
+          <t>Consolidate 3 Client Scope v1 drafts</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Prakhar</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Published catalogue ready for official release (Due Sept 14)</t>
+          <t>3 Scopes ready for technical feasibility review</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2280,17 +2280,17 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>S2.8</t>
+          <t>S2.7</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Finalize &amp; format **Capability Registry v1**</t>
+          <t>Finalize &amp; format **Product Catalogue v1**</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Prakhar</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Seed registry ready for official release (Due Sept 14)</t>
+          <t>Published catalogue ready for official release (Due Sept 14)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2337,27 +2337,27 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
+          <t>Compartment 1: Market, Intake &amp; Client POCs</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>S2.9</t>
+          <t>S2.8</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>**In-House LMS Architecture &amp; Data Schema Design**</t>
+          <t>Finalize &amp; format **Capability Registry v1**</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Shubham</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Tue, Sept 8 (Day 8)</t>
+          <t>Fri, Sept 11 (Day 11)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Technical architecture spec for replacing Graphy in Mr. Learn</t>
+          <t>Seed registry ready for official release (Due Sept 14)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2404,12 +2404,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>S2.10</t>
+          <t>S2.9</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>**In-House LMS Core Build (Part 1: Course &amp; Content Engine)**</t>
+          <t>**In-House LMS Architecture &amp; Data Schema Design**</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 11 (Day 11)</t>
+          <t>Tue, Sept 8 (Day 8)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>In-house course structure, modules &amp; video delivery service</t>
+          <t>Technical architecture spec for replacing Graphy in Mr. Learn</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2466,12 +2466,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>S2.11</t>
+          <t>S2.10</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Curate clean demo environment: **Learning Suite**</t>
+          <t>**In-House LMS Core Build (Part 1: Course &amp; Content Engine)**</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 9 (Day 9)</t>
+          <t>Fri, Sept 11 (Day 11)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Seeded with safe, client-presentable student data</t>
+          <t>In-house course structure, modules &amp; video delivery service</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2528,12 +2528,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>S2.12</t>
+          <t>S2.11</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Curate clean demo environment: **Sales CRM**</t>
+          <t>Curate clean demo environment: **Learning Suite**</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 10 (Day 10)</t>
+          <t>Wed, Sept 9 (Day 9)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Stripped of internal MAS lead data; clean CRM pipeline</t>
+          <t>Seeded with safe, client-presentable student data</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2590,22 +2590,22 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>S2.13</t>
+          <t>S2.12</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>**Demo #2: Learning Suite Walkthrough**</t>
+          <t>Curate clean demo environment: **Sales CRM**</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>**Wed, Sept 9 (Day 9)**</t>
+          <t>Thu, Sept 10 (Day 10)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>**Weekday baseline demo of Learning Suite**</t>
+          <t>Stripped of internal MAS lead data; clean CRM pipeline</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2647,27 +2647,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
+          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>S2.14</t>
+          <t>S2.13</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Identify idle, duplicate, orphaned cloud resources</t>
+          <t>**Demo #2: Learning Suite Walkthrough**</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Rohan</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Mon, Sept 7 (Day 7)</t>
+          <t>**Wed, Sept 9 (Day 9)**</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Cloud cleanup action list (disks, IPs, test VMs)</t>
+          <t>**Weekday baseline demo of Learning Suite**</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2714,12 +2714,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>S2.15</t>
+          <t>S2.14</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Clean up unused resources &amp; permissions in GCP/AWS</t>
+          <t>Identify idle, duplicate, orphaned cloud resources</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Tue, Sept 8 (Day 8)</t>
+          <t>Mon, Sept 7 (Day 7)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Reduced waste &amp; cleaner cloud estate</t>
+          <t>Cloud cleanup action list (disks, IPs, test VMs)</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2776,12 +2776,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>S2.16</t>
+          <t>S2.15</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Apply naming, ownership and cost tagging to cloud assets</t>
+          <t>Clean up unused resources &amp; permissions in GCP/AWS</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 9 (Day 9)</t>
+          <t>Tue, Sept 8 (Day 8)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Resources traceable by product and environment</t>
+          <t>Reduced waste &amp; cleaner cloud estate</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>S2.17</t>
+          <t>S2.16</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Prototype token &amp; latency tracking helper / middleware</t>
+          <t>Apply naming, ownership and cost tagging to cloud assets</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 10 (Day 10)</t>
+          <t>Wed, Sept 9 (Day 9)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Request-level token logging on suite endpoints</t>
+          <t>Resources traceable by product and environment</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2900,12 +2900,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>S2.18</t>
+          <t>S2.17</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Score collected departmental automation workflows</t>
+          <t>Prototype token &amp; latency tracking helper / middleware</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 11 (Day 11)</t>
+          <t>Thu, Sept 10 (Day 10)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Workflows ranked by effort, impact, hours saved</t>
+          <t>Request-level token logging on suite endpoints</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2962,22 +2962,22 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>S2.19</t>
+          <t>S2.18</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>**Full live pod rollout of Slack Standup Bot**</t>
+          <t>Score collected departmental automation workflows</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Rohan</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>**Mon, Sept 7 (Day 7)**</t>
+          <t>Fri, Sept 11 (Day 11)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>**100% daily standup updates captured via Slack DMs &amp; synced**</t>
+          <t>Workflows ranked by effort, impact, hours saved</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -3024,12 +3024,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>S2.20</t>
+          <t>S2.19</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>**Add /standup-notes &amp; weekend rollover handler**</t>
+          <t>**Full live pod rollout of Slack Standup Bot**</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>**Thu, Sept 10 (Day 10)**</t>
+          <t>**Mon, Sept 7 (Day 7)**</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>**Post-call highlight logger and weekend rollover features live**</t>
+          <t>**100% daily standup updates captured via Slack DMs &amp; synced**</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -3081,27 +3081,27 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
+          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>S2.21</t>
+          <t>S2.20</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Screen resumes &amp; interview QA Tester candidates</t>
+          <t>**Add /standup-notes &amp; weekend rollover handler**</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Gaurav</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 9 (Day 9)</t>
+          <t>**Thu, Sept 10 (Day 10)**</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>QA candidate shortlisted &amp; evaluated</t>
+          <t>**Post-call highlight logger and weekend rollover features live**</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -3148,12 +3148,12 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>S2.22</t>
+          <t>S2.21</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Screen resumes &amp; interview PM Intern candidates</t>
+          <t>Screen resumes &amp; interview QA Tester candidates</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>PM Intern candidate evaluated</t>
+          <t>QA candidate shortlisted &amp; evaluated</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -3210,12 +3210,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>S2.23</t>
+          <t>S2.22</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Extend offers for QA Tester and PM Intern</t>
+          <t>Screen resumes &amp; interview PM Intern candidates</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 11 (Day 11)</t>
+          <t>Wed, Sept 9 (Day 9)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3235,7 +3235,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Offers extended for Sept 21 onboarding</t>
+          <t>PM Intern candidate evaluated</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -3272,12 +3272,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>S2.24</t>
+          <t>S2.23</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Define GPU model-serving architecture with Sajan</t>
+          <t>Extend offers for QA Tester and PM Intern</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 10 (Day 10)</t>
+          <t>Fri, Sept 11 (Day 11)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>API vs Self-hosted cost comparison note</t>
+          <t>Offers extended for Sept 21 onboarding</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>S2.25</t>
+          <t>S2.24</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>**Weekly Review #2: Month 1 Mid-Point Sign-off**</t>
+          <t>Define GPU model-serving architecture with Sajan</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 11 (Day 11)</t>
+          <t>Thu, Sept 10 (Day 10)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Intake sign-off confirmed; LMS Build Part 1 progress review</t>
+          <t>API vs Self-hosted cost comparison note</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -3386,32 +3386,32 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Compartment 1: Market, Intake &amp; Client POCs</t>
+          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>S3.1</t>
+          <t>S2.25</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>**Publish Product Catalogue v1 (M5)**</t>
+          <t>**Weekly Review #2: Month 1 Mid-Point Sign-off**</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Prakhar</t>
+          <t>Gaurav</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>**Mon, Sept 14 (Day 14)**</t>
+          <t>Fri, Sept 11 (Day 11)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>**Catalogue v1 complete &amp; published for Business**</t>
+          <t>Intake sign-off confirmed; LMS Build Part 1 progress review</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -3458,17 +3458,17 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>S3.2</t>
+          <t>S3.1</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>**Publish Capability Registry v1 (M5)**</t>
+          <t>**Publish Product Catalogue v1 (M5)**</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Prakhar</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>**Registry v1 seeded &amp; published for Business**</t>
+          <t>**Catalogue v1 complete &amp; published for Business**</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -3520,22 +3520,22 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>S3.3</t>
+          <t>S3.2</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Conduct technical feasibility review on 3 client scopes</t>
+          <t>**Publish Capability Registry v1 (M5)**</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Shubham</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 16 (Day 16)</t>
+          <t>**Mon, Sept 14 (Day 14)**</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Feasibility note &amp; rough effort estimate per client</t>
+          <t>**Registry v1 seeded &amp; published for Business**</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3582,22 +3582,22 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>S3.4</t>
+          <t>S3.3</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Finalize written POC Scope: **Orane**</t>
+          <t>Conduct technical feasibility review on 3 client scopes</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 17 (Day 17)</t>
+          <t>Wed, Sept 16 (Day 16)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Written scope document ready for Business &amp; client sign-off</t>
+          <t>Feasibility note &amp; rough effort estimate per client</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3644,12 +3644,12 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>S3.5</t>
+          <t>S3.4</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Finalize written POC Scope: **College Vidya**</t>
+          <t>Finalize written POC Scope: **Orane**</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3706,12 +3706,12 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>S3.6</t>
+          <t>S3.5</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Finalize written POC Scope: **Chitkara**</t>
+          <t>Finalize written POC Scope: **College Vidya**</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 18 (Day 18)</t>
+          <t>Thu, Sept 17 (Day 17)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3768,12 +3768,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>S3.7</t>
+          <t>S3.6</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>**Secure 3 Accepted Written POC Scopes (M1)**</t>
+          <t>Finalize written POC Scope: **Chitkara**</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>**Sun, Sept 20 (Day 20)**</t>
+          <t>Fri, Sept 18 (Day 18)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>**3 Written POC scopes accepted by client and Business**</t>
+          <t>Written scope document ready for Business &amp; client sign-off</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3830,22 +3830,22 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>S3.8</t>
+          <t>S3.7</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Mandatory intake process enforcement on all new leads</t>
+          <t>**Secure 3 Accepted Written POC Scopes (M1)**</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Prakhar</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>**Sun, Sept 20 (Day 20)**</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>100% of new client requests enter through standard intake</t>
+          <t>**3 Written POC scopes accepted by client and Business**</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -3887,27 +3887,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
+          <t>Compartment 1: Market, Intake &amp; Client POCs</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>S3.9</t>
+          <t>S3.8</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>**In-House LMS Build (Part 2: Student OS &amp; Progress Tracking)**</t>
+          <t>Mandatory intake process enforcement on all new leads</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Shubham</t>
+          <t>Prakhar</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 16 (Day 16)</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Student profile, module progress &amp; analytics tracking module</t>
+          <t>100% of new client requests enter through standard intake</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -3954,12 +3954,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>S3.10</t>
+          <t>S3.9</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>**In-House LMS Integration with Mr. Learn &amp; Mr. Test**</t>
+          <t>**In-House LMS Build (Part 2: Student OS &amp; Progress Tracking)**</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 18 (Day 18)</t>
+          <t>Wed, Sept 16 (Day 16)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Working prototype connecting Mr. Learn UI to in-house LMS</t>
+          <t>Student profile, module progress &amp; analytics tracking module</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -4016,12 +4016,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>S3.11</t>
+          <t>S3.10</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Create short 15-min demo flow/script per suite</t>
+          <t>**In-House LMS Integration with Mr. Learn &amp; Mr. Test**</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 16 (Day 16)</t>
+          <t>Fri, Sept 18 (Day 18)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Business-ready demo flow &amp; narrative scripts</t>
+          <t>Working prototype connecting Mr. Learn UI to in-house LMS</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -4078,22 +4078,22 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>S3.12</t>
+          <t>S3.11</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>**Demo #3: Sales &amp; Admin Suite Walkthrough**</t>
+          <t>Create short 15-min demo flow/script per suite</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Prakhar</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>**Thu, Sept 17 (Day 17)**</t>
+          <t>Wed, Sept 16 (Day 16)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>**Weekday demo of Sales &amp; Admin Suite**</t>
+          <t>Business-ready demo flow &amp; narrative scripts</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -4140,22 +4140,22 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>S3.13</t>
+          <t>S3.12</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Start QA regression test suite on P0 products</t>
+          <t>**Demo #3: Sales &amp; Admin Suite Walkthrough**</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>QA / Tester</t>
+          <t>Prakhar</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 18 (Day 18)</t>
+          <t>**Thu, Sept 17 (Day 17)**</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Regression test cases drafted and executing</t>
+          <t>**Weekday demo of Sales &amp; Admin Suite**</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -4197,27 +4197,27 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
+          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>S3.14</t>
+          <t>S3.13</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Restructure cloud projects &amp; accounts where required</t>
+          <t>Start QA regression test suite on P0 products</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Rohan</t>
+          <t>QA / Tester</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Tue, Sept 15 (Day 15)</t>
+          <t>Fri, Sept 18 (Day 18)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Clean logical separation across GCP/AWS</t>
+          <t>Regression test cases drafted and executing</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -4264,12 +4264,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>S3.15</t>
+          <t>S3.14</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Separate dev / demo / production environments</t>
+          <t>Restructure cloud projects &amp; accounts where required</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -4279,7 +4279,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 17 (Day 17)</t>
+          <t>Tue, Sept 15 (Day 15)</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Isolated demo environment preventing test contamination</t>
+          <t>Clean logical separation across GCP/AWS</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -4326,12 +4326,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>S3.16</t>
+          <t>S3.15</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Select top 1 simple, high-value departmental workflow</t>
+          <t>Separate dev / demo / production environments</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 16 (Day 16)</t>
+          <t>Thu, Sept 17 (Day 17)</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Target automation selected for Month 1 build</t>
+          <t>Isolated demo environment preventing test contamination</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -4388,12 +4388,12 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>S3.17</t>
+          <t>S3.16</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Build &amp; test first internal automation workflow prototype</t>
+          <t>Select top 1 simple, high-value departmental workflow</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 18 (Day 18)</t>
+          <t>Wed, Sept 16 (Day 16)</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Core automation script/integration built</t>
+          <t>Target automation selected for Month 1 build</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -4450,12 +4450,12 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>S3.18</t>
+          <t>S3.17</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>**Switch on AI Cost Instrumentation Baseline (M4)**</t>
+          <t>Build &amp; test first internal automation workflow prototype</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>**Mon, Sept 21 (Day 21)**</t>
+          <t>Fri, Sept 18 (Day 18)</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>**Product-level token/API spend visible for live workloads**</t>
+          <t>Core automation script/integration built</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -4507,27 +4507,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
+          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>S3.19</t>
+          <t>S3.18</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Advance GPU compute/vendor discussions with Sajan</t>
+          <t>**Switch on AI Cost Instrumentation Baseline (M4)**</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Gaurav</t>
+          <t>Rohan</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 17 (Day 17)</t>
+          <t>**Mon, Sept 21 (Day 21)**</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Hardware spec options, vendor terms, and cost projection</t>
+          <t>**Product-level token/API spend visible for live workloads**</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -4574,12 +4574,12 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>S3.20</t>
+          <t>S3.19</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>**Weekly Product &amp; Capability Review #3 (8:00 PM)**</t>
+          <t>Advance GPU compute/vendor discussions with Sajan</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 18 (Day 18)</t>
+          <t>Thu, Sept 17 (Day 17)</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -4599,7 +4599,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Review minutes, LMS Prototype Part 2 preview &amp; ad-hoc audit</t>
+          <t>Hardware spec options, vendor terms, and cost projection</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4636,12 +4636,12 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>S3.21</t>
+          <t>S3.20</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>**Onboard QA Tester &amp; PM Intern (M8)**</t>
+          <t>**Weekly Product &amp; Capability Review #3 (8:00 PM)**</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>**Mon, Sept 21 (Day 21)**</t>
+          <t>Fri, Sept 18 (Day 18)</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>**QA active on P0 regression; Intern active on tasks**</t>
+          <t>Review minutes, LMS Prototype Part 2 preview &amp; ad-hoc audit</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -4688,32 +4688,32 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Compartment 1: Market, Intake &amp; Client POCs</t>
+          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>S4.1</t>
+          <t>S3.21</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Hand over accepted POC scopes to Tech Lead</t>
+          <t>**Onboard QA Tester &amp; PM Intern (M8)**</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Gaurav</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Tue, Sept 22 (Day 22)</t>
+          <t>**Mon, Sept 21 (Day 21)**</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Clear deployment handoff for Orane, CV, Chitkara</t>
+          <t>**QA active on P0 regression; Intern active on tasks**</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -4760,12 +4760,12 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>S4.2</t>
+          <t>S4.1</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Deploy PM Intern on catalogue &amp; client tracking</t>
+          <t>Hand over accepted POC scopes to Tech Lead</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 24 (Day 24)</t>
+          <t>Tue, Sept 22 (Day 22)</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -4785,7 +4785,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>PM Intern operational on tracking &amp; meeting logs</t>
+          <t>Clear deployment handoff for Orane, CV, Chitkara</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -4822,22 +4822,22 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>S4.3</t>
+          <t>S4.2</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Publish Month 2 Backlog (including Externalisation Gap Sheet)</t>
+          <t>Deploy PM Intern on catalogue &amp; client tracking</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Prakhar</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Sat, Sept 26 (Day 26)</t>
+          <t>Thu, Sept 24 (Day 24)</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Prioritized engineering sprint backlog for Month 2</t>
+          <t>PM Intern operational on tracking &amp; meeting logs</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -4879,27 +4879,27 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
+          <t>Compartment 1: Market, Intake &amp; Client POCs</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>S4.4</t>
+          <t>S4.3</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Execute full demo dry-runs with QA on both live suites</t>
+          <t>Publish Month 2 Backlog (including Externalisation Gap Sheet)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Shubham</t>
+          <t>Prakhar</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 23 (Day 23)</t>
+          <t>Sat, Sept 26 (Day 26)</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>End-to-end regression &amp; flow validation pass</t>
+          <t>Prioritized engineering sprint backlog for Month 2</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -4946,22 +4946,22 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>S4.5</t>
+          <t>S4.4</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>**Demo #4: Learning Suite Walkthrough (with LMS Prototype)**</t>
+          <t>Execute full demo dry-runs with QA on both live suites</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>**Thu, Sept 24 (Day 24)**</t>
+          <t>Wed, Sept 23 (Day 23)</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>**Weekday demo of Learning Suite with In-House LMS Preview**</t>
+          <t>End-to-end regression &amp; flow validation pass</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
@@ -5008,22 +5008,22 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>S4.6</t>
+          <t>S4.5</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Fix all remaining demo and staging edge cases</t>
+          <t>**Demo #4: Learning Suite Walkthrough (with LMS Prototype)**</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Rohan</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Thu, Sept 24 (Day 24)</t>
+          <t>**Thu, Sept 24 (Day 24)**</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Zero critical bugs; staging rock solid</t>
+          <t>**Weekday demo of Learning Suite with In-House LMS Preview**</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -5070,22 +5070,22 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>S4.7</t>
+          <t>S4.6</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>**P0 Stabilisation &amp; Demo Readiness Sign-Off (M2)**</t>
+          <t>Fix all remaining demo and staging edge cases</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Shubham</t>
+          <t>Rohan</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>**Fri, Sept 25 (Day 25)**</t>
+          <t>Thu, Sept 24 (Day 24)</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>**100% of P0 products demo-able on 24h notice; zero critical bugs**</t>
+          <t>Zero critical bugs; staging rock solid</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -5127,22 +5127,22 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
+          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>S4.8</t>
+          <t>S4.7</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>**Document final GCP + AWS architecture &amp; ownership**</t>
+          <t>**P0 Stabilisation &amp; Demo Readiness Sign-Off (M2)**</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Rohan</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Shared cloud infra map with cost attribution by product</t>
+          <t>**100% of P0 products demo-able on 24h notice; zero critical bugs**</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -5194,12 +5194,12 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>S4.9</t>
+          <t>S4.8</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Deploy &amp; test internal automation with actual department users</t>
+          <t>**Document final GCP + AWS architecture &amp; ownership**</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 25 (Day 25)</t>
+          <t>**Fri, Sept 25 (Day 25)**</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Live end-to-end workflow execution</t>
+          <t>Shared cloud infra map with cost attribution by product</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -5256,12 +5256,12 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>S4.10</t>
+          <t>S4.9</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Measure baseline vs post-automation hours saved per week</t>
+          <t>Deploy &amp; test internal automation with actual department users</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Mon, Sept 28 (Day 28)</t>
+          <t>Fri, Sept 25 (Day 25)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Measured internal service value metric</t>
+          <t>Live end-to-end workflow execution</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -5318,12 +5318,12 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>S4.11</t>
+          <t>S4.10</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>**Launch First Internal AI Automation Workflow Live (M7)**</t>
+          <t>Measure baseline vs post-automation hours saved per week</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>**Mon, Sept 28 (Day 28)**</t>
+          <t>Mon, Sept 28 (Day 28)</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>**Workflow live in production; weekly hours saved tracked**</t>
+          <t>Measured internal service value metric</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -5375,27 +5375,27 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
+          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>S4.12</t>
+          <t>S4.11</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>**Weekly Review #4: P0 Demo Readiness Sign-off (8:00 PM)**</t>
+          <t>**Launch First Internal AI Automation Workflow Live (M7)**</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Gaurav</t>
+          <t>Rohan</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Fri, Sept 25 (Day 25)</t>
+          <t>**Mon, Sept 28 (Day 28)**</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Review minutes, Demo sign-off &amp; LMS prototype verification</t>
+          <t>**Workflow live in production; weekly hours saved tracked**</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -5442,12 +5442,12 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>S4.13</t>
+          <t>S4.12</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>**Finalize September GPU / Compute Setup Track (M10)**</t>
+          <t>**Weekly Review #4: P0 Demo Readiness Sign-off (8:00 PM)**</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>**Wed, Sept 30 (Day 30)**</t>
+          <t>Fri, Sept 25 (Day 25)</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>**Compute option, vendor contact, architecture &amp; cost plan ready**</t>
+          <t>Review minutes, Demo sign-off &amp; LMS prototype verification</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
@@ -5504,17 +5504,17 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>S4.14</t>
+          <t>S4.13</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>**MAS AI Labs Website &amp; Info ID Live (M11)**</t>
+          <t>**Finalize September GPU / Compute Setup Track (M10)**</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Marketing / Vendor</t>
+          <t>Gaurav</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>**Website live + Info ID routed to named owner**</t>
+          <t>**Compute option, vendor contact, architecture &amp; cost plan ready**</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -5566,22 +5566,22 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>S4.15</t>
+          <t>S4.14</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Close 3 financial baselines (Revenue target, run-rate, hiring)</t>
+          <t>**MAS AI Labs Website &amp; Info ID Live (M11)**</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Gaurav</t>
+          <t>Marketing / Vendor</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Wed, Sept 30 (Day 30)</t>
+          <t>**Wed, Sept 30 (Day 30)**</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Closed financial baselines with Jitin Sir &amp; Pranab Sir</t>
+          <t>**Website live + Info ID routed to named owner**</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -5628,50 +5628,112 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
+          <t>S4.15</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Close 3 financial baselines (Revenue target, run-rate, hiring)</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Gaurav</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Wed, Sept 30 (Day 30)</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>[ ] Planned</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Closed financial baselines with Jitin Sir &amp; Pranab Sir</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
           <t>S4.16</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>**Publish Month-End Management Report &amp; Month 2 Backlog**</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>Gaurav</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>**Wed, Sept 30 (Day 30)**</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>[ ] Planned</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>[ ] Planned</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>**Comprehensive Month 1 closure report &amp; Month 2 plan**</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K84" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L84" s="2" t="inlineStr">
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -5688,7 +5750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -5699,7 +5761,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
@@ -6074,7 +6136,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>[!] Blocked</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -6089,7 +6151,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Need to discuss the artifacts required for capability mapping</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -6245,7 +6307,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -6260,7 +6322,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>working on bug hunterz pipeline migrating it to new email and also improving the pipeline</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -6270,7 +6332,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6391,27 +6453,27 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
+          <t>Compartment 2: Product, In-House LMS &amp; Demo Stabilisation</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>S1.12</t>
+          <t>S1.22</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Inventory current GCP projects, services &amp; VMs</t>
+          <t>Sales Suite technical documentation &amp; research plan</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Rohan</t>
+          <t>Shubham</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Thu, Sept 3 (Day 3)</t>
+          <t>Fri, Sept 4 (Day 4)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -6421,7 +6483,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Complete GCP infrastructure inventory with instance sizes</t>
+          <t>Technical architecture doc &amp; generalized setup plan</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -6453,12 +6515,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>S1.13</t>
+          <t>S1.12</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Inventory AWS accounts/services used by AI Labs</t>
+          <t>Inventory current GCP projects, services &amp; VMs</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -6468,7 +6530,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Fri, Sept 4 (Day 4)</t>
+          <t>Thu, Sept 3 (Day 3)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -6478,7 +6540,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Complete AWS inventory (S3, compute, IAM)</t>
+          <t>Complete GCP infrastructure inventory with instance sizes</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -6510,12 +6572,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>S1.14</t>
+          <t>S1.13</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Master inventory of AI/API keys, models &amp; endpoints</t>
+          <t>Inventory AWS accounts/services used by AI Labs</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -6535,7 +6597,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>All third-party AI keys mapped to product modules</t>
+          <t>Complete AWS inventory (S3, compute, IAM)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -6567,12 +6629,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>S1.15</t>
+          <t>S1.14</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Collect top repetitive workflows across MAS departments</t>
+          <t>Master inventory of AI/API keys, models &amp; endpoints</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -6592,7 +6654,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Departmental automation intake list (Problem $\rightarrow$ Effort $\rightarrow$ Value)</t>
+          <t>All third-party AI keys mapped to product modules</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -6624,32 +6686,32 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>S1.16</t>
+          <t>S1.15</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>**Build &amp; configure MAS Slack Standup Bot v1.0**</t>
+          <t>Collect top repetitive workflows across MAS departments</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Yashvi</t>
+          <t>Rohan</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>**Thu, Sept 3 (Day 3)**</t>
+          <t>Fri, Sept 4 (Day 4)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>**Personal DMs, dropdown modal, 7:45 PM summary &amp; 2-way sync**</t>
+          <t>Departmental automation intake list (Problem $\rightarrow$ Effort $\rightarrow$ Value)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -6681,12 +6743,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>S1.17</t>
+          <t>S1.16</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>**Test &amp; pilot Slack Standup Bot with core team**</t>
+          <t>**Build &amp; configure MAS Slack Standup Bot v1.0**</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -6696,7 +6758,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>**Fri, Sept 4 (Day 4)**</t>
+          <t>**Thu, Sept 3 (Day 3)**</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -6706,7 +6768,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>**Live test during Friday standup &amp; Friday review #1**</t>
+          <t>**Personal DMs, dropdown modal, 7:45 PM summary &amp; 2-way sync**</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -6716,7 +6778,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Need to discuss the artifacts required for capability mapping</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -6726,34 +6788,34 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
+          <t>Compartment 3: Cloud, Cost &amp; Internal Automation</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>S1.18</t>
+          <t>S1.17</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Kick off QA Tester (contract/2-mo) hiring</t>
+          <t>**Test &amp; pilot Slack Standup Bot with core team**</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Gaurav</t>
+          <t>Yashvi</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Tue, Sept 1 (Day 1)</t>
+          <t>**Fri, Sept 4 (Day 4)**</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -6763,7 +6825,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Active job description &amp; candidate pipeline with HR</t>
+          <t>**Live test during Friday standup &amp; Friday review #1**</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -6773,7 +6835,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Need to discuss the artifacts required for capability mapping</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -6783,7 +6845,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6795,12 +6857,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>S1.19</t>
+          <t>S1.18</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Kick off PM Intern (25 hrs/wk) hiring</t>
+          <t>Kick off QA Tester (contract/2-mo) hiring</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -6815,12 +6877,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Active job description &amp; candidate sourcing</t>
+          <t>Active job description &amp; candidate pipeline with HR</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -6852,12 +6914,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>S1.20</t>
+          <t>S1.19</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Initial September GPU/compute sync with Sajan</t>
+          <t>Kick off PM Intern (25 hrs/wk) hiring</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -6867,7 +6929,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Thu, Sept 3 (Day 3)</t>
+          <t>Tue, Sept 1 (Day 1)</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -6877,7 +6939,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Compute vendor contacts &amp; initial workload candidate list</t>
+          <t>Active job description &amp; candidate sourcing</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -6909,50 +6971,107 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
+          <t>S1.20</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Initial September GPU/compute sync with Sajan</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Gaurav</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Thu, Sept 3 (Day 3)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>[ ] Planned</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Compute vendor contacts &amp; initial workload candidate list</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Compartment 4: Leadership, Compute &amp; Enablers</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
           <t>S1.21</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>**Weekly Product &amp; Capability Review #1 (8:00 PM)**</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Gaurav</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Fri, Sept 4 (Day 4)</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>[ ] Planned</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>[ ] Planned</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Review minutes, Week 1 bug fix verification &amp; RAG audit</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>

</xml_diff>

<commit_message>
feat(rag): update RAG indicator mapping so In Progress and Planned are Yellow/Amber (🟡) while Completed is Green (🟢) and Blocked is Red (🔴)
</commit_message>
<xml_diff>
--- a/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
+++ b/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5425,7 @@
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5549,7 +5549,7 @@
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5933,7 +5933,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6275,7 +6275,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6389,7 +6389,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6446,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6560,7 +6560,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6617,7 +6617,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6959,7 +6959,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7016,7 +7016,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7214,7 +7214,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7385,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7499,7 +7499,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7613,7 +7613,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7727,7 +7727,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7898,7 +7898,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -7955,7 +7955,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8012,7 +8012,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8069,7 +8069,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8240,7 +8240,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8354,7 +8354,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8468,7 +8468,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8525,7 +8525,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8723,7 +8723,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8780,7 +8780,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9008,7 +9008,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9065,7 +9065,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9122,7 +9122,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9236,7 +9236,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9293,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9407,7 +9407,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9464,7 +9464,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9521,7 +9521,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9578,7 +9578,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9635,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9692,7 +9692,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9749,7 +9749,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -9863,7 +9863,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10004,7 +10004,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10061,7 +10061,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10118,7 +10118,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10175,7 +10175,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10232,7 +10232,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10289,7 +10289,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10403,7 +10403,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10460,7 +10460,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10574,7 +10574,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10631,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10688,7 +10688,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10745,7 +10745,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10802,7 +10802,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -10859,7 +10859,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(digest): remove stale blocker references and publish clean real-time pre-standup task summary
</commit_message>
<xml_diff>
--- a/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
+++ b/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
@@ -463,7 +463,7 @@
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Need to understand the deliverable</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Built &amp; configured with Socket Mode &amp; scheduler</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Need to discuss the artifacts required for capability mapping</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1628,12 +1628,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Live testing with pod members</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Need to discuss the artifacts required for capability mapping</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
@@ -5908,7 +5908,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -5965,7 +5965,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Need to understand the deliverable</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6773,12 +6773,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Built &amp; configured with Socket Mode &amp; scheduler</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Need to discuss the artifacts required for capability mapping</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -6788,7 +6788,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6830,12 +6830,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Live testing with pod members</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Need to discuss the artifacts required for capability mapping</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rag): standardize 4-color RAG (⚪ Not Started, 🟡 In Progress, 🔴 Blocked, 🟢 Completed) and highlight blocked task S1.6 under Yashvi
</commit_message>
<xml_diff>
--- a/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
+++ b/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5425,7 @@
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5549,7 +5549,7 @@
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5611,7 +5611,7 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5933,7 +5933,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6161,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6446,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6503,7 +6503,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6560,7 +6560,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6617,7 +6617,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6959,7 +6959,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7016,7 +7016,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7214,7 +7214,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7385,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7499,7 +7499,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7613,7 +7613,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7727,7 +7727,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7898,7 +7898,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -7955,7 +7955,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8012,7 +8012,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8069,7 +8069,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8240,7 +8240,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8354,7 +8354,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8468,7 +8468,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8525,7 +8525,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8723,7 +8723,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8780,7 +8780,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9008,7 +9008,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9065,7 +9065,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9122,7 +9122,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9236,7 +9236,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9293,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9407,7 +9407,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9464,7 +9464,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9521,7 +9521,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9578,7 +9578,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9635,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9692,7 +9692,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9749,7 +9749,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -9863,7 +9863,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10004,7 +10004,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10061,7 +10061,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10118,7 +10118,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10175,7 +10175,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10232,7 +10232,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10289,7 +10289,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10403,7 +10403,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10460,7 +10460,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10574,7 +10574,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10631,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10688,7 +10688,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10745,7 +10745,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10802,7 +10802,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -10859,7 +10859,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(standup): ingest Day 2 Google Meet notes, unblock resolved tasks, broadcast sleek highlights to #all-mas-ai-labs, and sync sprint tracker
</commit_message>
<xml_diff>
--- a/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
+++ b/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Creating client contact intake sheet in Google Sheet format</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Need to understand the deliverable</t>
+          <t>Aligned on Week 2 demo readiness; assigning component owners</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Email delivery bug fixed; info email account migrated; testing pipeline</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Sales Suite prototype presented (DB separation &amp; lead import); backend analysis underway</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Built &amp; configured with Socket Mode &amp; scheduler</t>
+          <t>Slack bot integrated with Gmail &amp; Gemini notes parsing</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Live testing with pod members</t>
+          <t>Live pilot testing with core team during daily standups</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -5861,7 +5861,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Creating client contact intake sheet in Google Sheet format</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Need to understand the deliverable</t>
+          <t>Aligned on Week 2 demo readiness; assigning component owners</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6317,7 +6317,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Email delivery bug fixed; info email account migrated; testing pipeline</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6478,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[-] In Progress</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -6488,7 +6488,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Sales Suite prototype presented (DB separation &amp; lead import); backend analysis underway</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Built &amp; configured with Socket Mode &amp; scheduler</t>
+          <t>Slack bot integrated with Gmail &amp; Gemini notes parsing</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Live testing with pod members</t>
+          <t>Live pilot testing with core team during daily standups</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(blockers): enforce automatic blocker reset when tasks are updated or resolved, preventing stale blockers from persisting across daily digests
</commit_message>
<xml_diff>
--- a/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
+++ b/sprint_execution/MAS_AI_LABS_SPRINT_TRACKER.xlsx
@@ -464,7 +464,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
@@ -636,7 +636,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Will start today</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Will start today</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Will start today</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[x] Completed</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Aligned on Week 2 demo readiness; assigning component owners</t>
+          <t>Need to update it at end of the month</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Need to discuss the artifacts required for capability mapping</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[x] Completed</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>working on bug hunterz pipeline migrating it to new email and also improving the pipeline</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[x] Completed</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[!] Blocked</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Slack bot integrated with Gmail &amp; Gemini notes parsing</t>
+          <t>slack bot formatting fixing in progress</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Live pilot testing with core team during daily standups</t>
+          <t>Testing daily summaries and improve the AI summarisation</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -5761,7 +5761,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Will start today</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Will start today</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Will start today</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -6136,7 +6136,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[x] Completed</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -6146,12 +6146,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Aligned on Week 2 demo readiness; assigning component owners</t>
+          <t>Need to update it at end of the month</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Need to discuss the artifacts required for capability mapping</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[x] Completed</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6250,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6322,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>working on bug hunterz pipeline migrating it to new email and also improving the pipeline</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[ ] Planned</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6478,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>[-] In Progress</t>
+          <t>[x] Completed</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6535,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>[ ] Planned</t>
+          <t>[!] Blocked</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6664,7 +6664,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>GPT credit exhausted</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Slack bot integrated with Gmail &amp; Gemini notes parsing</t>
+          <t>slack bot formatting fixing in progress</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Live pilot testing with core team during daily standups</t>
+          <t>Testing daily summaries and improve the AI summarisation</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">

</xml_diff>